<commit_message>
Voiles : aciers horizontaux HA10 face extérieure (poussée) et HA8 face intérieure
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KevyrhSMyW6Rq5jfFAg4co
</commit_message>
<xml_diff>
--- a/documents/DQE_Debourse_Voiles_Radier_170m.xlsx
+++ b/documents/DQE_Debourse_Voiles_Radier_170m.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Acier HA8 (voiles horiz., épingles, plantants en U e = 20 cm)</t>
+          <t>Acier HA8 (voiles horiz. face intérieure, épingles, plantants en U e = 20 cm)</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="D21" s="9">
-        <f>'Avant-metre'!$H$30</f>
+        <f>'Avant-metre'!$H$31</f>
         <v/>
       </c>
       <c r="E21" s="10">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Acier HA10 (radier longitudinal + chaises)</t>
+          <t>Acier HA10 (voiles horiz. face extérieure, radier longitudinal + chaises)</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="D22" s="9">
-        <f>'Avant-metre'!$H$31</f>
+        <f>'Avant-metre'!$H$32</f>
         <v/>
       </c>
       <c r="E22" s="10">
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="D23" s="9">
-        <f>'Avant-metre'!$H$32</f>
+        <f>'Avant-metre'!$H$33</f>
         <v/>
       </c>
       <c r="E23" s="10">
@@ -1374,45 +1374,52 @@
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="21" t="inlineStr">
         <is>
-          <t>• Plantants en U HA8 e = 20 cm : U ancré dans le radier, une jambe de 0,60 m dans chaque nappe du voile (jonction voile/radier).</t>
+          <t>• Voiles – aciers horizontaux : HA10 sur la face extérieure (reprise de la poussée) et HA8 sur la face intérieure, e = 20 cm.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="21" t="inlineStr">
         <is>
-          <t>• Béton fabriqué sur chantier à la bétonnière ; cure humide d'au moins 7 jours obligatoire (chaleur tropicale) ; bétonnage de préférence le matin.</t>
+          <t>• Plantants en U HA8 e = 20 cm : U ancré dans le radier, une jambe de 0,60 m dans chaque nappe du voile (jonction voile/radier).</t>
         </is>
       </c>
     </row>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="21" t="inlineStr">
         <is>
-          <t>• Fond de forme latéritique compacté à 95 % OPM ; purge des zones argileuses non comprise.</t>
+          <t>• Béton fabriqué sur chantier à la bétonnière ; cure humide d'au moins 7 jours obligatoire (chaleur tropicale) ; bétonnage de préférence le matin.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="24" customHeight="1">
       <c r="A40" s="21" t="inlineStr">
         <is>
+          <t>• Fond de forme latéritique compacté à 95 % OPM ; purge des zones argileuses non comprise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
           <t>• Prix de base indicatifs Abidjan 2026 – à actualiser selon les cotations fournisseurs (feuille « Hypotheses », cellules jaunes).</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="20" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="20" t="inlineStr">
         <is>
           <t>Établi par : Moulo Jean Claude</t>
         </is>
       </c>
-      <c r="F42" s="20" t="inlineStr">
+      <c r="F43" s="20" t="inlineStr">
         <is>
           <t>Visa / Approbation :</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="23">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A39:H39"/>
@@ -1422,6 +1429,7 @@
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A41:H41"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="A3:H3"/>
@@ -1797,7 +1805,7 @@
     <row r="22">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>Voiles – HA8 horizontaux, espacement (2 nappes)</t>
+          <t>Voiles – horizontaux HA10 ext. / HA8 int., espacement</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -2866,7 +2874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3390,27 +3398,27 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>V2</t>
+          <t>V2a</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Voiles – barres horizontales, 2 nappes</t>
+          <t>Voiles – barres horizontales, nappe EXTÉRIEURE (côté poussée)</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D24" s="26">
         <f>Hypotheses!$C$22</f>
         <v/>
       </c>
       <c r="E24" s="27">
-        <f>(ROUNDUP((Hypotheses!$C$10-Hypotheses!$C$14)/D24,0)+1)*2*Hypotheses!$C$9</f>
+        <f>(ROUNDUP((Hypotheses!$C$10-Hypotheses!$C$14)/D24,0)+1)*Hypotheses!$C$9</f>
         <v/>
       </c>
       <c r="F24" s="26">
-        <f>Hypotheses!$C$8-2*Hypotheses!$C$14+2*Hypotheses!$C$29+(ROUNDUP(Hypotheses!$C$8/Hypotheses!$C$32,0)-1)*Hypotheses!$C$31*8/1000</f>
+        <f>Hypotheses!$C$8-2*Hypotheses!$C$14+2*Hypotheses!$C$29+(ROUNDUP(Hypotheses!$C$8/Hypotheses!$C$32,0)-1)*Hypotheses!$C$31*10/1000</f>
         <v/>
       </c>
       <c r="G24" s="28">
@@ -3418,36 +3426,39 @@
         <v/>
       </c>
       <c r="H24" s="25">
-        <f>G24*Hypotheses!$C$33</f>
+        <f>G24*Hypotheses!$C$34</f>
         <v/>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>Nb filants = (H/esp + 1) × 2 × Nv ; L = L + retours + recouvrements 50Ø</t>
+          <t>Nb filants = (H/esp + 1) × Nv ; L = L + retours + recouvrements 50Ø – HA10 à cause de la poussée</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>V3</t>
+          <t>V2b</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Voiles – épingles de liaison des nappes</t>
+          <t>Voiles – barres horizontales, nappe INTÉRIEURE</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D25" s="26" t="inlineStr"/>
+      <c r="D25" s="26">
+        <f>Hypotheses!$C$22</f>
+        <v/>
+      </c>
       <c r="E25" s="27">
-        <f>ROUNDUP(Hypotheses!$C$9*Hypotheses!$C$8*Hypotheses!$C$10*Hypotheses!$C$27,0)</f>
+        <f>(ROUNDUP((Hypotheses!$C$10-Hypotheses!$C$14)/D25,0)+1)*Hypotheses!$C$9</f>
         <v/>
       </c>
       <c r="F25" s="26">
-        <f>Hypotheses!$C$11-2*Hypotheses!$C$14+2*0.10</f>
+        <f>Hypotheses!$C$8-2*Hypotheses!$C$14+2*Hypotheses!$C$29+(ROUNDUP(Hypotheses!$C$8/Hypotheses!$C$32,0)-1)*Hypotheses!$C$31*8/1000</f>
         <v/>
       </c>
       <c r="G25" s="28">
@@ -3460,34 +3471,31 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>4 u/m² ; L = e − 2 enr. + 2 crochets</t>
+          <t>Nb filants = (H/esp + 1) × Nv ; L = L + retours + recouvrements 50Ø</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>V4</t>
+          <t>V3</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Plantants en U (jonction voile / radier)</t>
+          <t>Voiles – épingles de liaison des nappes</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D26" s="26">
-        <f>Hypotheses!$C$25</f>
-        <v/>
-      </c>
+      <c r="D26" s="26" t="inlineStr"/>
       <c r="E26" s="27">
-        <f>(ROUNDUP(Hypotheses!$C$8/D26,0)+1)*Hypotheses!$C$9</f>
+        <f>ROUNDUP(Hypotheses!$C$9*Hypotheses!$C$8*Hypotheses!$C$10*Hypotheses!$C$27,0)</f>
         <v/>
       </c>
       <c r="F26" s="26">
-        <f>2*(Hypotheses!$C$26+Hypotheses!$C$13-Hypotheses!$C$14)+(Hypotheses!$C$11-2*Hypotheses!$C$14)</f>
+        <f>Hypotheses!$C$11-2*Hypotheses!$C$14+2*0.10</f>
         <v/>
       </c>
       <c r="G26" s="28">
@@ -3500,34 +3508,34 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>U ancré dans le radier, 2 jambes de 0,60 m dans le voile (une par nappe)</t>
+          <t>4 u/m² ; L = e − 2 enr. + 2 crochets</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>V4</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Radier – barres transversales, 2 nappes</t>
+          <t>Plantants en U (jonction voile / radier)</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D27" s="26">
-        <f>Hypotheses!$C$23</f>
+        <f>Hypotheses!$C$25</f>
         <v/>
       </c>
       <c r="E27" s="27">
-        <f>(ROUNDUP(Hypotheses!$C$8/D27,0)+1)*2</f>
+        <f>(ROUNDUP(Hypotheses!$C$8/D27,0)+1)*Hypotheses!$C$9</f>
         <v/>
       </c>
       <c r="F27" s="26">
-        <f>Hypotheses!$C$12-2*Hypotheses!$C$14+2*Hypotheses!$C$29</f>
+        <f>2*(Hypotheses!$C$26+Hypotheses!$C$13-Hypotheses!$C$14)+(Hypotheses!$C$11-2*Hypotheses!$C$14)</f>
         <v/>
       </c>
       <c r="G27" s="28">
@@ -3535,39 +3543,39 @@
         <v/>
       </c>
       <c r="H27" s="25">
-        <f>G27*Hypotheses!$C$35</f>
+        <f>G27*Hypotheses!$C$33</f>
         <v/>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>(L/esp + 1) × 2 nappes ; L = B − 2 enr. + 2 retours</t>
+          <t>U ancré dans le radier, 2 jambes de 0,60 m dans le voile (une par nappe)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Radier – barres longitudinales, 2 nappes</t>
+          <t>Radier – barres transversales, 2 nappes</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D28" s="26">
-        <f>Hypotheses!$C$24</f>
+        <f>Hypotheses!$C$23</f>
         <v/>
       </c>
       <c r="E28" s="27">
-        <f>(ROUNDUP((Hypotheses!$C$12-2*Hypotheses!$C$14)/D28,0)+1)*2</f>
+        <f>(ROUNDUP(Hypotheses!$C$8/D28,0)+1)*2</f>
         <v/>
       </c>
       <c r="F28" s="26">
-        <f>Hypotheses!$C$8-2*Hypotheses!$C$14+2*Hypotheses!$C$29+(ROUNDUP(Hypotheses!$C$8/Hypotheses!$C$32,0)-1)*Hypotheses!$C$31*10/1000</f>
+        <f>Hypotheses!$C$12-2*Hypotheses!$C$14+2*Hypotheses!$C$29</f>
         <v/>
       </c>
       <c r="G28" s="28">
@@ -3575,36 +3583,39 @@
         <v/>
       </c>
       <c r="H28" s="25">
-        <f>G28*Hypotheses!$C$34</f>
+        <f>G28*Hypotheses!$C$35</f>
         <v/>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>Nb filants = (B/esp + 1) × 2 ; L avec recouvrements 50Ø</t>
+          <t>(L/esp + 1) × 2 nappes ; L = B − 2 enr. + 2 retours</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Radier – chaises support nappe supérieure</t>
+          <t>Radier – barres longitudinales, 2 nappes</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="D29" s="26" t="inlineStr"/>
+      <c r="D29" s="26">
+        <f>Hypotheses!$C$24</f>
+        <v/>
+      </c>
       <c r="E29" s="27">
-        <f>ROUNDUP(Hypotheses!$C$8*Hypotheses!$C$12*Hypotheses!$C$28,0)</f>
+        <f>(ROUNDUP((Hypotheses!$C$12-2*Hypotheses!$C$14)/D29,0)+1)*2</f>
         <v/>
       </c>
       <c r="F29" s="26">
-        <f>0.60</f>
+        <f>Hypotheses!$C$8-2*Hypotheses!$C$14+2*Hypotheses!$C$29+(ROUNDUP(Hypotheses!$C$8/Hypotheses!$C$32,0)-1)*Hypotheses!$C$31*10/1000</f>
         <v/>
       </c>
       <c r="G29" s="28">
@@ -3617,32 +3628,51 @@
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
+          <t>Nb filants = (B/esp + 1) × 2 ; L avec recouvrements 50Ø</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Radier – chaises support nappe supérieure</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D30" s="26" t="inlineStr"/>
+      <c r="E30" s="27">
+        <f>ROUNDUP(Hypotheses!$C$8*Hypotheses!$C$12*Hypotheses!$C$28,0)</f>
+        <v/>
+      </c>
+      <c r="F30" s="26">
+        <f>0.60</f>
+        <v/>
+      </c>
+      <c r="G30" s="28">
+        <f>E30*F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="25">
+        <f>G30*Hypotheses!$C$34</f>
+        <v/>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
           <t>1 u/m²</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>TOTAL HA8 (kg nets)</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="29">
-        <f>SUMIF($C$23:$C$29,8,$H$23:$H$29)</f>
-        <v/>
-      </c>
-      <c r="I30" s="14" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>TOTAL HA10 (kg nets)</t>
+          <t>TOTAL HA8 (kg nets)</t>
         </is>
       </c>
       <c r="B31" s="6" t="n"/>
@@ -3652,7 +3682,7 @@
       <c r="F31" s="6" t="n"/>
       <c r="G31" s="6" t="n"/>
       <c r="H31" s="29">
-        <f>SUMIF($C$23:$C$29,10,$H$23:$H$29)</f>
+        <f>SUMIF($C$23:$C$30,8,$H$23:$H$30)</f>
         <v/>
       </c>
       <c r="I31" s="14" t="inlineStr"/>
@@ -3660,7 +3690,7 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>TOTAL HA12 (kg nets)</t>
+          <t>TOTAL HA10 (kg nets)</t>
         </is>
       </c>
       <c r="B32" s="6" t="n"/>
@@ -3670,7 +3700,7 @@
       <c r="F32" s="6" t="n"/>
       <c r="G32" s="6" t="n"/>
       <c r="H32" s="29">
-        <f>SUMIF($C$23:$C$29,12,$H$23:$H$29)</f>
+        <f>SUMIF($C$23:$C$30,10,$H$23:$H$30)</f>
         <v/>
       </c>
       <c r="I32" s="14" t="inlineStr"/>
@@ -3678,7 +3708,7 @@
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>TOTAL ACIERS (kg nets)</t>
+          <t>TOTAL HA12 (kg nets)</t>
         </is>
       </c>
       <c r="B33" s="6" t="n"/>
@@ -3688,15 +3718,15 @@
       <c r="F33" s="6" t="n"/>
       <c r="G33" s="6" t="n"/>
       <c r="H33" s="29">
-        <f>SUM(H30:H32)</f>
+        <f>SUMIF($C$23:$C$30,12,$H$23:$H$30)</f>
         <v/>
       </c>
       <c r="I33" s="14" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr">
-        <is>
-          <t>Ratio acier (kg/m³ de béton armé)</t>
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL ACIERS (kg nets)</t>
         </is>
       </c>
       <c r="B34" s="6" t="n"/>
@@ -3705,97 +3735,82 @@
       <c r="E34" s="6" t="n"/>
       <c r="F34" s="6" t="n"/>
       <c r="G34" s="6" t="n"/>
-      <c r="H34" s="30">
-        <f>H33/('Avant-metre'!$H$13+'Avant-metre'!$H$14)</f>
-        <v/>
-      </c>
-      <c r="I34" s="8" t="inlineStr">
+      <c r="H34" s="29">
+        <f>SUM(H31:H33)</f>
+        <v/>
+      </c>
+      <c r="I34" s="14" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>Ratio acier (kg/m³ de béton armé)</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="30">
+        <f>H34/('Avant-metre'!$H$13+'Avant-metre'!$H$14)</f>
+        <v/>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
         <is>
           <t>Ordre de grandeur usuel voiles/radiers : 60 à 120 kg/m³</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>6. VÉRIFICATION DES SECTIONS MINIMALES (EC2 §9.6 et §9.3 / BAEL)</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="6" t="n"/>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="6" t="n"/>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="6" t="n"/>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="6" t="n"/>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Élément</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Vérification</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr"/>
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>Conclusion</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>Voile</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>As,v fourni (HA12, 2 nappes)</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>mm²/m</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>2 × π×12²/4 / s</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="27">
-        <f>2*PI()*12^2/4/Hypotheses!$C$21</f>
-        <v/>
-      </c>
-      <c r="I38" s="8">
-        <f>IF(H38&gt;=H39,"OK","À renforcer")</f>
-        <v/>
       </c>
     </row>
     <row r="39">
@@ -3806,7 +3821,7 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>As,v,min = 0,002·Ac</t>
+          <t>As,v fourni (HA12, 2 nappes)</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -3816,17 +3831,20 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>EC2 §9.6.2(1)</t>
+          <t>2 × π×12²/4 / s</t>
         </is>
       </c>
       <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n"/>
       <c r="G39" s="6" t="n"/>
       <c r="H39" s="27">
-        <f>0.002*Hypotheses!$C$11*1000*1000</f>
-        <v/>
-      </c>
-      <c r="I39" s="8" t="inlineStr"/>
+        <f>2*PI()*12^2/4/Hypotheses!$C$21</f>
+        <v/>
+      </c>
+      <c r="I39" s="8">
+        <f>IF(H39&gt;=H40,"OK","À renforcer")</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3836,7 +3854,7 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>As,h fourni (HA8, 2 nappes)</t>
+          <t>As,v,min = 0,002·Ac</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -3846,20 +3864,17 @@
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>2 × π×8²/4 / s</t>
+          <t>EC2 §9.6.2(1)</t>
         </is>
       </c>
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="6" t="n"/>
       <c r="G40" s="6" t="n"/>
       <c r="H40" s="27">
-        <f>2*PI()*8^2/4/Hypotheses!$C$22</f>
-        <v/>
-      </c>
-      <c r="I40" s="8">
-        <f>IF(H40&gt;=H41,"OK","À renforcer")</f>
-        <v/>
-      </c>
+        <f>0.002*Hypotheses!$C$11*1000*1000</f>
+        <v/>
+      </c>
+      <c r="I40" s="8" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3869,7 +3884,7 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>As,h,min = max(25 % As,v ; 0,001·Ac)</t>
+          <t>As,h fourni (HA10 ext. + HA8 int.)</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -3879,27 +3894,30 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>EC2 §9.6.3(1)</t>
+          <t>(π×10²/4 + π×8²/4) / s</t>
         </is>
       </c>
       <c r="E41" s="6" t="n"/>
       <c r="F41" s="6" t="n"/>
       <c r="G41" s="6" t="n"/>
       <c r="H41" s="27">
-        <f>MAX(0.25*H38,0.001*Hypotheses!$C$11*1e6)</f>
-        <v/>
-      </c>
-      <c r="I41" s="8" t="inlineStr"/>
+        <f>(PI()*10^2/4+PI()*8^2/4)/Hypotheses!$C$22</f>
+        <v/>
+      </c>
+      <c r="I41" s="8">
+        <f>IF(H41&gt;=H42,"OK","À renforcer")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>Radier</t>
+          <t>Voile</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>As transv. fourni par nappe (HA12)</t>
+          <t>As,h,min = max(25 % As,v ; 0,001·Ac)</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -3909,20 +3927,17 @@
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>π×12²/4 / s</t>
+          <t>EC2 §9.6.3(1)</t>
         </is>
       </c>
       <c r="E42" s="6" t="n"/>
       <c r="F42" s="6" t="n"/>
       <c r="G42" s="6" t="n"/>
       <c r="H42" s="27">
-        <f>PI()*12^2/4/Hypotheses!$C$23</f>
-        <v/>
-      </c>
-      <c r="I42" s="8">
-        <f>IF(H42&gt;=H43,"OK","À renforcer")</f>
-        <v/>
-      </c>
+        <f>MAX(0.25*H39,0.001*Hypotheses!$C$11*1e6)</f>
+        <v/>
+      </c>
+      <c r="I42" s="8" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3932,7 +3947,7 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>As,min = max(0,26·fctm/fyk ; 0,0013)·b·d</t>
+          <t>As transv. fourni par nappe (HA12)</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
@@ -3942,17 +3957,20 @@
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>C25/30 : fctm = 2,6 MPa ; d = e − enr. − Ø/2</t>
+          <t>π×12²/4 / s</t>
         </is>
       </c>
       <c r="E43" s="6" t="n"/>
       <c r="F43" s="6" t="n"/>
       <c r="G43" s="6" t="n"/>
       <c r="H43" s="27">
-        <f>MAX(0.26*2.6/500,0.0013)*1000*(Hypotheses!$C$13-Hypotheses!$C$14-0.006)*1000</f>
-        <v/>
-      </c>
-      <c r="I43" s="8" t="inlineStr"/>
+        <f>PI()*12^2/4/Hypotheses!$C$23</f>
+        <v/>
+      </c>
+      <c r="I43" s="8">
+        <f>IF(H43&gt;=H44,"OK","À renforcer")</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3962,7 +3980,7 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>As long. fourni par nappe (HA10)</t>
+          <t>As,min = max(0,26·fctm/fyk ; 0,0013)·b·d</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
@@ -3972,63 +3990,93 @@
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>π×10²/4 / s</t>
+          <t>C25/30 : fctm = 2,6 MPa ; d = e − enr. − Ø/2</t>
         </is>
       </c>
       <c r="E44" s="6" t="n"/>
       <c r="F44" s="6" t="n"/>
       <c r="G44" s="6" t="n"/>
       <c r="H44" s="27">
+        <f>MAX(0.26*2.6/500,0.0013)*1000*(Hypotheses!$C$13-Hypotheses!$C$14-0.006)*1000</f>
+        <v/>
+      </c>
+      <c r="I44" s="8" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Radier</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>As long. fourni par nappe (HA10)</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>mm²/m</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>π×10²/4 / s</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="27">
         <f>PI()*10^2/4/Hypotheses!$C$24</f>
         <v/>
       </c>
-      <c r="I44" s="8">
-        <f>IF(H44&gt;=0.2*H42,"OK (≥ 20 % As princ.)","À renforcer")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="I45" s="8">
+        <f>IF(H45&gt;=0.2*H43,"OK (≥ 20 % As princ.)","À renforcer")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>NB : ces vérifications portent uniquement sur les sections minimales et les espacements réglementaires. Les sections réelles doivent être confirmées par une note de calcul (poussée des terres/eau sur voiles, réaction du sol latéritique sous radier).</t>
         </is>
       </c>
     </row>
-    <row r="47"/>
+    <row r="48"/>
   </sheetData>
   <mergeCells count="32">
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="D12:G12"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="D8:G8"/>
     <mergeCell ref="D39:G39"/>
-    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="A35:G35"/>
     <mergeCell ref="A18:I18"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="D42:G42"/>
-    <mergeCell ref="D38:G38"/>
     <mergeCell ref="A21:I21"/>
     <mergeCell ref="D14:G14"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="D44:G44"/>
-    <mergeCell ref="A30:G30"/>
     <mergeCell ref="D19:G19"/>
     <mergeCell ref="D10:G10"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="D40:G40"/>
+    <mergeCell ref="D45:G45"/>
     <mergeCell ref="D13:G13"/>
-    <mergeCell ref="A46:I47"/>
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="D41:G41"/>
     <mergeCell ref="D17:G17"/>
     <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A36:I36"/>
     <mergeCell ref="D16:G16"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="D43:G43"/>
     <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A47:I48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>